<commit_message>
feat: complete brand blue UI upgrade, custom dropdown popups, modal alignment, and performance optimizations
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -2859,7 +2859,11 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>KAVIN019</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3368,7 +3372,11 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>SAJAN_VENKAT</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3445,7 +3453,11 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LeueJEWPmY</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3522,7 +3534,11 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>STALIN_A</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3707,7 +3723,11 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>_Tamilarasan</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -5261,7 +5281,11 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr"/>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>GAgrm4ykwn</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -5311,7 +5335,11 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E183" t="inlineStr"/>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Smitha_M</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -5523,7 +5551,11 @@
           <t>II</t>
         </is>
       </c>
-      <c r="E191" t="inlineStr"/>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>VANITHA_E</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -6383,7 +6415,11 @@
           <t>III</t>
         </is>
       </c>
-      <c r="E223" t="inlineStr"/>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Aadhish_sb</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -6946,7 +6982,11 @@
           <t>III</t>
         </is>
       </c>
-      <c r="E244" t="inlineStr"/>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>prasath_2628_</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -7320,7 +7360,11 @@
           <t>III</t>
         </is>
       </c>
-      <c r="E258" t="inlineStr"/>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>rahul_kumar42</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -8010,7 +8054,11 @@
           <t>IV</t>
         </is>
       </c>
-      <c r="E284" t="inlineStr"/>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>kamal_vishnu</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -8141,7 +8189,11 @@
           <t>IV</t>
         </is>
       </c>
-      <c r="E289" t="inlineStr"/>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>KAVIN-V</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -8322,7 +8374,11 @@
           <t>IV</t>
         </is>
       </c>
-      <c r="E296" t="inlineStr"/>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>sathishsaravanan_33</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">

</xml_diff>